<commit_message>
Refactor app.py to improve user instructions and remove API key check; update binary files
</commit_message>
<xml_diff>
--- a/output/listings.xlsx
+++ b/output/listings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:AD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,12 +572,12 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1804 - 1048 BROADVIEW AVENUE</t>
+          <t>106 - 80 ORCHID PLACE DRIVE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TORONTO</t>
+          <t>TORONTO (MALVERN)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -587,59 +587,55 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>M4K2B8</t>
+          <t>M1B0C4</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LAURA ISOBEL CATALANO</t>
+          <t>CHRISTINE HAZEL BOLAND</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>RE/MAX HALLMARK REALTY LTD.</t>
+          <t>CROWN NORTH REALTY INC.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>$449,000</t>
+          <t>$509,000</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>43.6851857</t>
+          <t>43.79363</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-79.3567489</t>
+          <t>-79.23575</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>E13517800</t>
+          <t>E12998328</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>500 - 599</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>LAMINATE, TILE</t>
-        </is>
-      </c>
+          <t>700-799</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>CENTRAL AIR CONDITIONING</t>
@@ -647,7 +643,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>COIL FAN, FORCED AIR, (NATURAL GAS)</t>
+          <t>FORCED AIR (NATURAL GAS)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -668,18 +664,18 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>APARTMENT</t>
+          <t>ROW / TOWNHOUSE</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
-          <t>500 - 599 SQFT</t>
+          <t>700-799 SQFT</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>BROADVIEW NORTH</t>
+          <t>MALVERN</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -688,149 +684,285 @@
         </is>
       </c>
       <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0 TO 5 YEARS</t>
+        </is>
+      </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>$2532.12</t>
+          <t>$2,360</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1 HOUR</t>
+          <t>79 DAYS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
+          <t>1804 - 1048 BROADVIEW AVENUE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TORONTO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ONTARIO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>M4K2B8</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>LAURA ISOBEL CATALANO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>RE/MAX HALLMARK REALTY LTD.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>$449,000</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>43.6851857</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>-79.3567489</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>E13517800</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>500 - 599</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>LAMINATE, TILE</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>CENTRAL AIR CONDITIONING</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>COIL FAN, FORCED AIR, (NATURAL GAS)</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>UNDERGROUND, GARAGE</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SINGLE FAMILY</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>APARTMENT</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>500 - 599 SQFT</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>BROADVIEW NORTH</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>CONDOMINIUM/STRATA</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>0 TO 5 YEARS</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>$2532.12</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>1 HOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>206 - 1960 QUEEN STREET</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>TORONTO (THE BEACHES)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>ONTARIO</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>M4L 1H8</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>AEAZ BATHIA</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>RE/MAX ACE REALTY INC., BROKERAGE</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>$625,000</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>43.669766</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>-79.3020091</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>E13517746</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>600-699</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>LAMINATE, TILE</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>CENTRAL AIR CONDITIONING</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>FORCED AIR (NATURAL GAS)</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
         <is>
           <t>UNDERGROUND, GARAGE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>SINGLE FAMILY</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>APARTMENT</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr">
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr">
         <is>
           <t>600-699 SQFT</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>THE BEACHES</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>CONDOMINIUM/STRATA</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr">
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr">
         <is>
           <t>0 TO 5 YEARS</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>$4,331.26</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>59 MINUTES</t>
         </is>

</xml_diff>